<commit_message>
Set D shift to 12:00-20:00 in attendance sheets
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LsGdck9uUBqMn7Bw6wMhA5
</commit_message>
<xml_diff>
--- a/Personel_Devam_Cizelgesi_Eylul_2026_AYSENUR_YILMAZ.xlsx
+++ b/Personel_Devam_Cizelgesi_Eylul_2026_AYSENUR_YILMAZ.xlsx
@@ -1196,13 +1196,21 @@
       <c r="B15" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C15" s="28" t="n"/>
+      <c r="C15" s="28" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
       <c r="D15" s="6" t="n"/>
       <c r="E15" s="6" t="n"/>
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="n"/>
       <c r="H15" s="6" t="n"/>
-      <c r="I15" s="28" t="n"/>
+      <c r="I15" s="28" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
       <c r="J15" s="6" t="n"/>
       <c r="K15" s="7" t="n"/>
     </row>
@@ -1232,13 +1240,21 @@
       <c r="B17" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="C17" s="28" t="n"/>
+      <c r="C17" s="28" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
       <c r="D17" s="6" t="n"/>
       <c r="E17" s="6" t="n"/>
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="6" t="n"/>
       <c r="H17" s="6" t="n"/>
-      <c r="I17" s="28" t="n"/>
+      <c r="I17" s="28" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
       <c r="J17" s="9" t="n"/>
       <c r="K17" s="10" t="n"/>
     </row>
@@ -1246,13 +1262,21 @@
       <c r="B18" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="C18" s="28" t="n"/>
+      <c r="C18" s="28" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
       <c r="D18" s="6" t="n"/>
       <c r="E18" s="6" t="n"/>
       <c r="F18" s="6" t="n"/>
       <c r="G18" s="6" t="n"/>
       <c r="H18" s="6" t="n"/>
-      <c r="I18" s="28" t="n"/>
+      <c r="I18" s="28" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
       <c r="J18" s="9" t="n"/>
       <c r="K18" s="10" t="n"/>
     </row>
@@ -1304,13 +1328,21 @@
       <c r="B21" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="C21" s="28" t="n"/>
+      <c r="C21" s="28" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
       <c r="D21" s="6" t="n"/>
       <c r="E21" s="6" t="n"/>
       <c r="F21" s="6" t="n"/>
       <c r="G21" s="6" t="n"/>
       <c r="H21" s="6" t="n"/>
-      <c r="I21" s="28" t="n"/>
+      <c r="I21" s="28" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
       <c r="J21" s="9" t="n"/>
       <c r="K21" s="10" t="n"/>
     </row>
@@ -1318,13 +1350,21 @@
       <c r="B22" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="C22" s="28" t="n"/>
+      <c r="C22" s="28" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
       <c r="D22" s="6" t="n"/>
       <c r="E22" s="6" t="n"/>
       <c r="F22" s="6" t="n"/>
       <c r="G22" s="6" t="n"/>
       <c r="H22" s="6" t="n"/>
-      <c r="I22" s="28" t="n"/>
+      <c r="I22" s="28" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
       <c r="J22" s="9" t="n"/>
       <c r="K22" s="10" t="n"/>
     </row>
@@ -1332,13 +1372,21 @@
       <c r="B23" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="C23" s="28" t="n"/>
+      <c r="C23" s="28" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
       <c r="D23" s="6" t="n"/>
       <c r="E23" s="6" t="n"/>
       <c r="F23" s="6" t="n"/>
       <c r="G23" s="6" t="n"/>
       <c r="H23" s="6" t="n"/>
-      <c r="I23" s="28" t="n"/>
+      <c r="I23" s="28" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
       <c r="J23" s="9" t="n"/>
       <c r="K23" s="10" t="n"/>
     </row>
@@ -1368,13 +1416,21 @@
       <c r="B25" s="8" t="n">
         <v>11</v>
       </c>
-      <c r="C25" s="28" t="n"/>
+      <c r="C25" s="28" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
       <c r="D25" s="6" t="n"/>
       <c r="E25" s="6" t="n"/>
       <c r="F25" s="6" t="n"/>
       <c r="G25" s="6" t="n"/>
       <c r="H25" s="6" t="n"/>
-      <c r="I25" s="28" t="n"/>
+      <c r="I25" s="28" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
       <c r="J25" s="9" t="n"/>
       <c r="K25" s="10" t="n"/>
     </row>
@@ -1448,13 +1504,21 @@
       <c r="B29" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="C29" s="28" t="n"/>
+      <c r="C29" s="28" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
       <c r="D29" s="6" t="n"/>
       <c r="E29" s="6" t="n"/>
       <c r="F29" s="6" t="n"/>
       <c r="G29" s="6" t="n"/>
       <c r="H29" s="6" t="n"/>
-      <c r="I29" s="28" t="n"/>
+      <c r="I29" s="28" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
       <c r="J29" s="9" t="n"/>
       <c r="K29" s="10" t="n"/>
     </row>
@@ -1462,13 +1526,21 @@
       <c r="B30" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="C30" s="28" t="n"/>
+      <c r="C30" s="28" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
       <c r="D30" s="6" t="n"/>
       <c r="E30" s="6" t="n"/>
       <c r="F30" s="6" t="n"/>
       <c r="G30" s="6" t="n"/>
       <c r="H30" s="6" t="n"/>
-      <c r="I30" s="28" t="n"/>
+      <c r="I30" s="28" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
       <c r="J30" s="9" t="n"/>
       <c r="K30" s="10" t="n"/>
     </row>
@@ -1540,13 +1612,21 @@
       <c r="B35" s="8" t="n">
         <v>21</v>
       </c>
-      <c r="C35" s="28" t="n"/>
+      <c r="C35" s="28" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
       <c r="D35" s="6" t="n"/>
       <c r="E35" s="6" t="n"/>
       <c r="F35" s="6" t="n"/>
       <c r="G35" s="6" t="n"/>
       <c r="H35" s="6" t="n"/>
-      <c r="I35" s="28" t="n"/>
+      <c r="I35" s="28" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
       <c r="J35" s="9" t="n"/>
       <c r="K35" s="10" t="n"/>
     </row>

</xml_diff>